<commit_message>
feat: add module 3 pretest/posttest links
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_ลิงก์เอกสารและแบบทดสอบ.xlsx
+++ b/TFT_ลิงก์เอกสารและแบบทดสอบ.xlsx
@@ -871,8 +871,16 @@
           <t>Pretest</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>https://forms.gle/QB1JpfsKPLfj33y58</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>ได้รับลิงก์แล้ว (2569-09-27)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" s="8">
       <c r="A13" s="2" t="n">
@@ -903,8 +911,16 @@
           <t>Posttest</t>
         </is>
       </c>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="3" t="n"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>https://forms.gle/y3tkxJGyNQUFFMAf9</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>ได้รับลิงก์แล้ว (2569-09-27)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1870,27 +1886,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add module 2 pretest/posttest links
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TFT_ลิงก์เอกสารและแบบทดสอบ.xlsx
+++ b/TFT_ลิงก์เอกสารและแบบทดสอบ.xlsx
@@ -767,8 +767,16 @@
           <t>Pretest</t>
         </is>
       </c>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>https://forms.gle/qRUuf6EK7tWr1phPA</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>ได้รับลิงก์แล้ว (2569-09-27)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -799,8 +807,16 @@
           <t>Posttest</t>
         </is>
       </c>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>https://forms.gle/mNCoDUN5osWNwKjVA</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>ได้รับลิงก์แล้ว (2569-09-27)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="25.5" customHeight="1" s="8">
       <c r="A11" s="2" t="n">
@@ -1885,30 +1901,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>